<commit_message>
fix: update botanical name formatting and use JPG logo for PDF
- Updated formatting: species capitalized when no variant, lowercase with variant
- Examples: Acer Campestre (no variant) vs Acer campestre 'Red Shine' (with variant)
- Changed PDF logo from PNG to JPG (Papervale_LogoMark_Colour_RGB.jpg)
- Regenerated all availability files with updated formatting
</commit_message>
<xml_diff>
--- a/files/availability-list-2026.xlsx
+++ b/files/availability-list-2026.xlsx
@@ -501,7 +501,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Abies alba</t>
+          <t>Abies Alba</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -534,7 +534,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Abies concolor</t>
+          <t>Abies Concolor</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -567,7 +567,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Abies concolor</t>
+          <t>Abies Concolor</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -600,7 +600,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Abies fraseri</t>
+          <t>Abies Fraseri</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -633,7 +633,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Abies grandis</t>
+          <t>Abies Grandis</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -666,7 +666,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Abies grandis</t>
+          <t>Abies Grandis</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -699,7 +699,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Abies grandis</t>
+          <t>Abies Grandis</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -732,7 +732,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Abies koreana</t>
+          <t>Abies Koreana</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -765,7 +765,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Abies koreana</t>
+          <t>Abies Koreana</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -798,7 +798,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Abies koreana</t>
+          <t>Abies Koreana</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -831,7 +831,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Abies koreana</t>
+          <t>Abies Koreana</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -864,7 +864,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Abies lasiocarpa</t>
+          <t>Abies Lasiocarpa</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -897,7 +897,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Abies nobilis</t>
+          <t>Abies Nobilis</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -930,7 +930,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Abies nordmanniana</t>
+          <t>Abies Nordmanniana</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -963,7 +963,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Abies nordmanniana</t>
+          <t>Abies Nordmanniana</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -996,7 +996,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Abies nordmanniana</t>
+          <t>Abies Nordmanniana</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1029,7 +1029,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Abies pinsapo</t>
+          <t>Abies Pinsapo</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1062,7 +1062,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Abies pinsapo</t>
+          <t>Abies Pinsapo</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1095,7 +1095,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Acacia dealbata</t>
+          <t>Acacia Dealbata</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1128,7 +1128,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Acacia melanoxylon</t>
+          <t>Acacia Melanoxylon</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1232,7 +1232,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Acer buergerianum</t>
+          <t>Acer Buergerianum</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1270,7 +1270,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Acer buergerianum</t>
+          <t>Acer Buergerianum</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1303,7 +1303,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Acer campestre</t>
+          <t>Acer Campestre</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1341,7 +1341,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Acer campestre</t>
+          <t>Acer Campestre</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1379,7 +1379,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Acer campestre</t>
+          <t>Acer Campestre</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1417,7 +1417,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Acer campestre</t>
+          <t>Acer Campestre</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1450,7 +1450,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Acer campestre</t>
+          <t>Acer Campestre</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1483,7 +1483,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Acer campestre</t>
+          <t>Acer Campestre</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -1805,7 +1805,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Acer carpinifolium</t>
+          <t>Acer Carpinifolium</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -1838,7 +1838,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Acer davidii</t>
+          <t>Acer Davidii</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -1871,7 +1871,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Acer davidii</t>
+          <t>Acer Davidii</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -1909,7 +1909,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Acer davidii</t>
+          <t>Acer Davidii</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -1947,7 +1947,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Acer davidii</t>
+          <t>Acer Davidii</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -1985,7 +1985,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Acer davidii</t>
+          <t>Acer Davidii</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -2492,7 +2492,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Acer ginnala</t>
+          <t>Acer Ginnala</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -2525,7 +2525,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Acer ginnala</t>
+          <t>Acer Ginnala</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -2563,7 +2563,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Acer griseum</t>
+          <t>Acer Griseum</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -2596,7 +2596,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Acer griseum</t>
+          <t>Acer Griseum</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -2629,7 +2629,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Acer griseum</t>
+          <t>Acer Griseum</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -2662,7 +2662,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Acer monspessulanum</t>
+          <t>Acer Monspessulanum</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -2695,7 +2695,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Acer monspessulanum</t>
+          <t>Acer Monspessulanum</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -2870,7 +2870,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Acer palmatum</t>
+          <t>Acer Palmatum</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
@@ -2936,7 +2936,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Acer palmatum</t>
+          <t>Acer Palmatum</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
@@ -3002,7 +3002,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Acer plat.</t>
+          <t>Acer Plat.</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
@@ -3035,7 +3035,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Acer plat.</t>
+          <t>Acer Plat.</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
@@ -3073,7 +3073,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Acer plat.</t>
+          <t>Acer Plat.</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
@@ -3111,7 +3111,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Acer plat.</t>
+          <t>Acer Plat.</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
@@ -3149,7 +3149,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Acer plat.</t>
+          <t>Acer Plat.</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
@@ -3187,7 +3187,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Acer plat.</t>
+          <t>Acer Plat.</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
@@ -3225,7 +3225,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Acer plat.</t>
+          <t>Acer Plat.</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
@@ -3263,7 +3263,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Acer plat.</t>
+          <t>Acer Plat.</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
@@ -3874,7 +3874,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>Acer pseudoplatanus</t>
+          <t>Acer Pseudoplatanus</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
@@ -3907,7 +3907,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>Acer pseudoplatanus</t>
+          <t>Acer Pseudoplatanus</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
@@ -3945,7 +3945,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>Acer pseudoplatanus</t>
+          <t>Acer Pseudoplatanus</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
@@ -3983,7 +3983,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>Acer pseudoplatanus</t>
+          <t>Acer Pseudoplatanus</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
@@ -4021,7 +4021,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>Acer pseudoplatanus</t>
+          <t>Acer Pseudoplatanus</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
@@ -4059,7 +4059,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>Acer pseudoplatanus</t>
+          <t>Acer Pseudoplatanus</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
@@ -4097,7 +4097,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>Acer pseudoplatanus</t>
+          <t>Acer Pseudoplatanus</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
@@ -4130,7 +4130,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>Acer pseudoplatanus</t>
+          <t>Acer Pseudoplatanus</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
@@ -4315,7 +4315,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>Acer rubrum</t>
+          <t>Acer Rubrum</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
@@ -4348,7 +4348,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>Acer rubrum</t>
+          <t>Acer Rubrum</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
@@ -4386,7 +4386,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>Acer rubrum</t>
+          <t>Acer Rubrum</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
@@ -4424,7 +4424,7 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>Acer rubrum</t>
+          <t>Acer Rubrum</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
@@ -5017,7 +5017,7 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>Acer saccharinum</t>
+          <t>Acer Saccharinum</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
@@ -5050,7 +5050,7 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>Acer saccharinum</t>
+          <t>Acer Saccharinum</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
@@ -5088,7 +5088,7 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>Acer saccharinum</t>
+          <t>Acer Saccharinum</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
@@ -5126,7 +5126,7 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>Acer saccharinum</t>
+          <t>Acer Saccharinum</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
@@ -5164,7 +5164,7 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>Acer saccharinum</t>
+          <t>Acer Saccharinum</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
@@ -5202,7 +5202,7 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>Acer saccharinum</t>
+          <t>Acer Saccharinum</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
@@ -5240,7 +5240,7 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>Acer saccharinum</t>
+          <t>Acer Saccharinum</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
@@ -5278,7 +5278,7 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>Aesculus hippocastanum</t>
+          <t>Aesculus Hippocastanum</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
@@ -5316,7 +5316,7 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>Aesculus hippocastanum</t>
+          <t>Aesculus Hippocastanum</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
@@ -5349,7 +5349,7 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>Aesculus hippocastanum</t>
+          <t>Aesculus Hippocastanum</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
@@ -5415,7 +5415,7 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>Aesculus indica</t>
+          <t>Aesculus Indica</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
@@ -5481,7 +5481,7 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>Albizia julibrissin</t>
+          <t>Albizia Julibrissin</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
@@ -5514,7 +5514,7 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>Alnus cordata</t>
+          <t>Alnus Cordata</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
@@ -5547,7 +5547,7 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>Alnus cordata</t>
+          <t>Alnus Cordata</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
@@ -5585,7 +5585,7 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>Alnus cordata</t>
+          <t>Alnus Cordata</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
@@ -5623,7 +5623,7 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>Alnus cordata</t>
+          <t>Alnus Cordata</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
@@ -5661,7 +5661,7 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>Alnus glutinosa</t>
+          <t>Alnus Glutinosa</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
@@ -5699,7 +5699,7 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>Alnus glutinosa</t>
+          <t>Alnus Glutinosa</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
@@ -5775,7 +5775,7 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>Alnus glutinosa</t>
+          <t>Alnus Glutinosa</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
@@ -5808,7 +5808,7 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>Alnus glutinosa</t>
+          <t>Alnus Glutinosa</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
@@ -5846,7 +5846,7 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>Alnus glutinosa</t>
+          <t>Alnus Glutinosa</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
@@ -5884,7 +5884,7 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>Alnus glutinosa</t>
+          <t>Alnus Glutinosa</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
@@ -5922,7 +5922,7 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>Alnus glutinosa</t>
+          <t>Alnus Glutinosa</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
@@ -5960,7 +5960,7 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>Alnus glutinosa</t>
+          <t>Alnus Glutinosa</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
@@ -6178,7 +6178,7 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>Alnus x</t>
+          <t>Alnus X</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>Alnus x</t>
+          <t>Alnus X</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
@@ -6419,7 +6419,7 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>Amelanchier canadensis</t>
+          <t>Amelanchier Canadensis</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
@@ -6485,7 +6485,7 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>Amelanchier lamarckii</t>
+          <t>Amelanchier Lamarckii</t>
         </is>
       </c>
       <c r="C171" t="inlineStr">
@@ -6518,7 +6518,7 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>Amelanchier lamarckii</t>
+          <t>Amelanchier Lamarckii</t>
         </is>
       </c>
       <c r="C172" t="inlineStr">
@@ -6551,7 +6551,7 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>Amelanchier lamarckii</t>
+          <t>Amelanchier Lamarckii</t>
         </is>
       </c>
       <c r="C173" t="inlineStr">
@@ -6584,7 +6584,7 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>Amelanchier lamarckii</t>
+          <t>Amelanchier Lamarckii</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
@@ -6622,7 +6622,7 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>Amelanchier lamarckii</t>
+          <t>Amelanchier Lamarckii</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
@@ -6655,7 +6655,7 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>Amelanchier lamarckii</t>
+          <t>Amelanchier Lamarckii</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
@@ -6693,7 +6693,7 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>Amelanchier lamarckii</t>
+          <t>Amelanchier Lamarckii</t>
         </is>
       </c>
       <c r="C177" t="inlineStr">
@@ -6731,7 +6731,7 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>Amelanchier lamarckii</t>
+          <t>Amelanchier Lamarckii</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
@@ -6769,7 +6769,7 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>Amelanchier lamarckii</t>
+          <t>Amelanchier Lamarckii</t>
         </is>
       </c>
       <c r="C179" t="inlineStr">
@@ -6807,7 +6807,7 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>Aralia elata</t>
+          <t>Aralia Elata</t>
         </is>
       </c>
       <c r="C180" t="inlineStr">
@@ -6840,7 +6840,7 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>Aralia elata</t>
+          <t>Aralia Elata</t>
         </is>
       </c>
       <c r="C181" t="inlineStr">
@@ -6873,7 +6873,7 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>Aralia elata</t>
+          <t>Aralia Elata</t>
         </is>
       </c>
       <c r="C182" t="inlineStr">
@@ -6906,7 +6906,7 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>Araucaria araucana</t>
+          <t>Araucaria Araucana</t>
         </is>
       </c>
       <c r="C183" t="inlineStr">
@@ -6939,7 +6939,7 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>Arbutus unedo</t>
+          <t>Arbutus Unedo</t>
         </is>
       </c>
       <c r="C184" t="inlineStr">
@@ -6977,7 +6977,7 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>Arbutus unedo</t>
+          <t>Arbutus Unedo</t>
         </is>
       </c>
       <c r="C185" t="inlineStr">
@@ -7195,7 +7195,7 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>Betula albosinensis</t>
+          <t>Betula Albosinensis</t>
         </is>
       </c>
       <c r="C191" t="inlineStr">
@@ -7233,7 +7233,7 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>Betula ermanii</t>
+          <t>Betula Ermanii</t>
         </is>
       </c>
       <c r="C192" t="inlineStr">
@@ -7266,7 +7266,7 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>Betula ermanii</t>
+          <t>Betula Ermanii</t>
         </is>
       </c>
       <c r="C193" t="inlineStr">
@@ -7299,7 +7299,7 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>Betula nigra</t>
+          <t>Betula Nigra</t>
         </is>
       </c>
       <c r="C194" t="inlineStr">
@@ -7337,7 +7337,7 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>Betula nigra</t>
+          <t>Betula Nigra</t>
         </is>
       </c>
       <c r="C195" t="inlineStr">
@@ -7375,7 +7375,7 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>Betula nigra</t>
+          <t>Betula Nigra</t>
         </is>
       </c>
       <c r="C196" t="inlineStr">
@@ -7413,7 +7413,7 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>Betula nigra</t>
+          <t>Betula Nigra</t>
         </is>
       </c>
       <c r="C197" t="inlineStr">
@@ -7446,7 +7446,7 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>Betula papyrifera</t>
+          <t>Betula Papyrifera</t>
         </is>
       </c>
       <c r="C198" t="inlineStr">
@@ -7479,7 +7479,7 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>Betula papyrifera</t>
+          <t>Betula Papyrifera</t>
         </is>
       </c>
       <c r="C199" t="inlineStr">
@@ -7512,7 +7512,7 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>Betula papyrifera</t>
+          <t>Betula Papyrifera</t>
         </is>
       </c>
       <c r="C200" t="inlineStr">
@@ -7550,7 +7550,7 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>Betula pendula</t>
+          <t>Betula Pendula</t>
         </is>
       </c>
       <c r="C201" t="inlineStr">
@@ -7583,7 +7583,7 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>Betula pendula</t>
+          <t>Betula Pendula</t>
         </is>
       </c>
       <c r="C202" t="inlineStr">
@@ -7616,7 +7616,7 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>Betula pendula</t>
+          <t>Betula Pendula</t>
         </is>
       </c>
       <c r="C203" t="inlineStr">
@@ -7654,7 +7654,7 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>Betula pendula</t>
+          <t>Betula Pendula</t>
         </is>
       </c>
       <c r="C204" t="inlineStr">
@@ -7692,7 +7692,7 @@
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>Betula pendula</t>
+          <t>Betula Pendula</t>
         </is>
       </c>
       <c r="C205" t="inlineStr">
@@ -7730,7 +7730,7 @@
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>Betula pendula</t>
+          <t>Betula Pendula</t>
         </is>
       </c>
       <c r="C206" t="inlineStr">
@@ -7768,7 +7768,7 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>Betula pendula</t>
+          <t>Betula Pendula</t>
         </is>
       </c>
       <c r="C207" t="inlineStr">
@@ -7806,7 +7806,7 @@
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>Betula pendula</t>
+          <t>Betula Pendula</t>
         </is>
       </c>
       <c r="C208" t="inlineStr">
@@ -7844,7 +7844,7 @@
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>Betula pendula</t>
+          <t>Betula Pendula</t>
         </is>
       </c>
       <c r="C209" t="inlineStr">
@@ -7882,7 +7882,7 @@
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>Betula pendula</t>
+          <t>Betula Pendula</t>
         </is>
       </c>
       <c r="C210" t="inlineStr">
@@ -7920,7 +7920,7 @@
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>Betula pendula</t>
+          <t>Betula Pendula</t>
         </is>
       </c>
       <c r="C211" t="inlineStr">
@@ -7953,7 +7953,7 @@
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>Betula pendula</t>
+          <t>Betula Pendula</t>
         </is>
       </c>
       <c r="C212" t="inlineStr">
@@ -7991,7 +7991,7 @@
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>Betula pendula</t>
+          <t>Betula Pendula</t>
         </is>
       </c>
       <c r="C213" t="inlineStr">
@@ -8029,7 +8029,7 @@
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>Betula pendula</t>
+          <t>Betula Pendula</t>
         </is>
       </c>
       <c r="C214" t="inlineStr">
@@ -8199,7 +8199,7 @@
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>Betula pendula</t>
+          <t>Betula Pendula</t>
         </is>
       </c>
       <c r="C219" t="inlineStr">
@@ -8232,7 +8232,7 @@
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>Betula pendula</t>
+          <t>Betula Pendula</t>
         </is>
       </c>
       <c r="C220" t="inlineStr">
@@ -8265,7 +8265,7 @@
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>Betula pendula</t>
+          <t>Betula Pendula</t>
         </is>
       </c>
       <c r="C221" t="inlineStr">
@@ -8303,7 +8303,7 @@
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>Betula pendula</t>
+          <t>Betula Pendula</t>
         </is>
       </c>
       <c r="C222" t="inlineStr">
@@ -8440,7 +8440,7 @@
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>Betula pubescens</t>
+          <t>Betula Pubescens</t>
         </is>
       </c>
       <c r="C226" t="inlineStr">
@@ -8473,7 +8473,7 @@
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>Betula pubescens</t>
+          <t>Betula Pubescens</t>
         </is>
       </c>
       <c r="C227" t="inlineStr">
@@ -8511,7 +8511,7 @@
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>Betula pubescens</t>
+          <t>Betula Pubescens</t>
         </is>
       </c>
       <c r="C228" t="inlineStr">
@@ -8544,7 +8544,7 @@
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>Betula pubescens</t>
+          <t>Betula Pubescens</t>
         </is>
       </c>
       <c r="C229" t="inlineStr">
@@ -8582,7 +8582,7 @@
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>Betula pubescens</t>
+          <t>Betula Pubescens</t>
         </is>
       </c>
       <c r="C230" t="inlineStr">
@@ -8620,7 +8620,7 @@
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>Betula pubescens</t>
+          <t>Betula Pubescens</t>
         </is>
       </c>
       <c r="C231" t="inlineStr">
@@ -8658,7 +8658,7 @@
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>Betula pubescens</t>
+          <t>Betula Pubescens</t>
         </is>
       </c>
       <c r="C232" t="inlineStr">
@@ -9008,7 +9008,7 @@
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>Betula utilis</t>
+          <t>Betula Utilis</t>
         </is>
       </c>
       <c r="C242" t="inlineStr">
@@ -9041,7 +9041,7 @@
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>Betula utilis</t>
+          <t>Betula Utilis</t>
         </is>
       </c>
       <c r="C243" t="inlineStr">
@@ -9074,7 +9074,7 @@
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>Betula utilis</t>
+          <t>Betula Utilis</t>
         </is>
       </c>
       <c r="C244" t="inlineStr">
@@ -9855,7 +9855,7 @@
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>Carpinus betulus</t>
+          <t>Carpinus Betulus</t>
         </is>
       </c>
       <c r="C266" t="inlineStr">
@@ -9893,7 +9893,7 @@
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>Carpinus betulus</t>
+          <t>Carpinus Betulus</t>
         </is>
       </c>
       <c r="C267" t="inlineStr">
@@ -9931,7 +9931,7 @@
       </c>
       <c r="B268" t="inlineStr">
         <is>
-          <t>Carpinus betulus</t>
+          <t>Carpinus Betulus</t>
         </is>
       </c>
       <c r="C268" t="inlineStr">
@@ -9964,7 +9964,7 @@
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>Carpinus betulus</t>
+          <t>Carpinus Betulus</t>
         </is>
       </c>
       <c r="C269" t="inlineStr">
@@ -10002,7 +10002,7 @@
       </c>
       <c r="B270" t="inlineStr">
         <is>
-          <t>Carpinus betulus</t>
+          <t>Carpinus Betulus</t>
         </is>
       </c>
       <c r="C270" t="inlineStr">
@@ -10040,7 +10040,7 @@
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>Carpinus betulus</t>
+          <t>Carpinus Betulus</t>
         </is>
       </c>
       <c r="C271" t="inlineStr">
@@ -10078,7 +10078,7 @@
       </c>
       <c r="B272" t="inlineStr">
         <is>
-          <t>Carpinus betulus</t>
+          <t>Carpinus Betulus</t>
         </is>
       </c>
       <c r="C272" t="inlineStr">
@@ -10116,7 +10116,7 @@
       </c>
       <c r="B273" t="inlineStr">
         <is>
-          <t>Carpinus betulus</t>
+          <t>Carpinus Betulus</t>
         </is>
       </c>
       <c r="C273" t="inlineStr">
@@ -10154,7 +10154,7 @@
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>Carpinus japonica</t>
+          <t>Carpinus Japonica</t>
         </is>
       </c>
       <c r="C274" t="inlineStr">
@@ -10187,7 +10187,7 @@
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>Carpinus japonica</t>
+          <t>Carpinus Japonica</t>
         </is>
       </c>
       <c r="C275" t="inlineStr">
@@ -10220,7 +10220,7 @@
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>Carya illinoinensis</t>
+          <t>Carya Illinoinensis</t>
         </is>
       </c>
       <c r="C276" t="inlineStr">
@@ -10253,7 +10253,7 @@
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>Carya ovata</t>
+          <t>Carya Ovata</t>
         </is>
       </c>
       <c r="C277" t="inlineStr">
@@ -10286,7 +10286,7 @@
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>Castanea sativa</t>
+          <t>Castanea Sativa</t>
         </is>
       </c>
       <c r="C278" t="inlineStr">
@@ -10319,7 +10319,7 @@
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>Castanea sativa</t>
+          <t>Castanea Sativa</t>
         </is>
       </c>
       <c r="C279" t="inlineStr">
@@ -10357,7 +10357,7 @@
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>Catalpa bignonioides</t>
+          <t>Catalpa Bignonioides</t>
         </is>
       </c>
       <c r="C280" t="inlineStr">
@@ -10390,7 +10390,7 @@
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>Catalpa bignonioides</t>
+          <t>Catalpa Bignonioides</t>
         </is>
       </c>
       <c r="C281" t="inlineStr">
@@ -10428,7 +10428,7 @@
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>Catalpa bignonioides</t>
+          <t>Catalpa Bignonioides</t>
         </is>
       </c>
       <c r="C282" t="inlineStr">
@@ -10461,7 +10461,7 @@
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>Catalpa bignonioides</t>
+          <t>Catalpa Bignonioides</t>
         </is>
       </c>
       <c r="C283" t="inlineStr">
@@ -10499,7 +10499,7 @@
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>Catalpa bignonioides</t>
+          <t>Catalpa Bignonioides</t>
         </is>
       </c>
       <c r="C284" t="inlineStr">
@@ -10537,7 +10537,7 @@
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>Catalpa bignonioides</t>
+          <t>Catalpa Bignonioides</t>
         </is>
       </c>
       <c r="C285" t="inlineStr">
@@ -10575,7 +10575,7 @@
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>Catalpa bignonioides</t>
+          <t>Catalpa Bignonioides</t>
         </is>
       </c>
       <c r="C286" t="inlineStr">
@@ -10646,7 +10646,7 @@
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>Cedrus atlantica</t>
+          <t>Cedrus Atlantica</t>
         </is>
       </c>
       <c r="C288" t="inlineStr">
@@ -10679,7 +10679,7 @@
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>Cedrus atlantica</t>
+          <t>Cedrus Atlantica</t>
         </is>
       </c>
       <c r="C289" t="inlineStr">
@@ -10717,7 +10717,7 @@
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>Cedrus atlantica</t>
+          <t>Cedrus Atlantica</t>
         </is>
       </c>
       <c r="C290" t="inlineStr">
@@ -10750,7 +10750,7 @@
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>Cedrus atlantica</t>
+          <t>Cedrus Atlantica</t>
         </is>
       </c>
       <c r="C291" t="inlineStr">
@@ -10783,7 +10783,7 @@
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>Cedrus deodara</t>
+          <t>Cedrus Deodara</t>
         </is>
       </c>
       <c r="C292" t="inlineStr">
@@ -10816,7 +10816,7 @@
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>Cedrus deodara</t>
+          <t>Cedrus Deodara</t>
         </is>
       </c>
       <c r="C293" t="inlineStr">
@@ -10849,7 +10849,7 @@
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>Cedrus libani</t>
+          <t>Cedrus Libani</t>
         </is>
       </c>
       <c r="C294" t="inlineStr">
@@ -10882,7 +10882,7 @@
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>Celtis sinensis</t>
+          <t>Celtis Sinensis</t>
         </is>
       </c>
       <c r="C295" t="inlineStr">
@@ -10915,7 +10915,7 @@
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>Cercidiphyllum japonicum</t>
+          <t>Cercidiphyllum Japonicum</t>
         </is>
       </c>
       <c r="C296" t="inlineStr">
@@ -10953,7 +10953,7 @@
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>Cercidiphyllum japonicum</t>
+          <t>Cercidiphyllum Japonicum</t>
         </is>
       </c>
       <c r="C297" t="inlineStr">
@@ -10991,7 +10991,7 @@
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>Cercidiphyllum japonicum</t>
+          <t>Cercidiphyllum Japonicum</t>
         </is>
       </c>
       <c r="C298" t="inlineStr">
@@ -11024,7 +11024,7 @@
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>Cercidiphyllum japonicum</t>
+          <t>Cercidiphyllum Japonicum</t>
         </is>
       </c>
       <c r="C299" t="inlineStr">
@@ -11057,7 +11057,7 @@
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>Chamaecyparis l.</t>
+          <t>Chamaecyparis L.</t>
         </is>
       </c>
       <c r="C300" t="inlineStr">
@@ -11090,7 +11090,7 @@
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>Chamaecyparis lawonsonia</t>
+          <t>Chamaecyparis Lawonsonia</t>
         </is>
       </c>
       <c r="C301" t="inlineStr">
@@ -11189,7 +11189,7 @@
       </c>
       <c r="B304" t="inlineStr">
         <is>
-          <t>Cladrastis kentukea</t>
+          <t>Cladrastis Kentukea</t>
         </is>
       </c>
       <c r="C304" t="inlineStr">
@@ -11222,7 +11222,7 @@
       </c>
       <c r="B305" t="inlineStr">
         <is>
-          <t>Cladrastis kentukea</t>
+          <t>Cladrastis Kentukea</t>
         </is>
       </c>
       <c r="C305" t="inlineStr">
@@ -11255,7 +11255,7 @@
       </c>
       <c r="B306" t="inlineStr">
         <is>
-          <t>Cordyline australis</t>
+          <t>Cordyline Australis</t>
         </is>
       </c>
       <c r="C306" t="inlineStr">
@@ -11288,7 +11288,7 @@
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>Cornus controversa</t>
+          <t>Cornus Controversa</t>
         </is>
       </c>
       <c r="C307" t="inlineStr">
@@ -11359,7 +11359,7 @@
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>Cornus florida</t>
+          <t>Cornus Florida</t>
         </is>
       </c>
       <c r="C309" t="inlineStr">
@@ -11491,7 +11491,7 @@
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>Cornus kousa</t>
+          <t>Cornus Kousa</t>
         </is>
       </c>
       <c r="C313" t="inlineStr">
@@ -11590,7 +11590,7 @@
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>Cornus kousa</t>
+          <t>Cornus Kousa</t>
         </is>
       </c>
       <c r="C316" t="inlineStr">
@@ -11623,7 +11623,7 @@
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>Cornus kousa</t>
+          <t>Cornus Kousa</t>
         </is>
       </c>
       <c r="C317" t="inlineStr">
@@ -11656,7 +11656,7 @@
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t>Cornus mas</t>
+          <t>Cornus Mas</t>
         </is>
       </c>
       <c r="C318" t="inlineStr">
@@ -11689,7 +11689,7 @@
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>Cornus mas</t>
+          <t>Cornus Mas</t>
         </is>
       </c>
       <c r="C319" t="inlineStr">
@@ -11722,7 +11722,7 @@
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>Cornus mas</t>
+          <t>Cornus Mas</t>
         </is>
       </c>
       <c r="C320" t="inlineStr">
@@ -11755,7 +11755,7 @@
       </c>
       <c r="B321" t="inlineStr">
         <is>
-          <t>Cornus mas</t>
+          <t>Cornus Mas</t>
         </is>
       </c>
       <c r="C321" t="inlineStr">
@@ -11793,7 +11793,7 @@
       </c>
       <c r="B322" t="inlineStr">
         <is>
-          <t>Cornus wilsoniana</t>
+          <t>Cornus Wilsoniana</t>
         </is>
       </c>
       <c r="C322" t="inlineStr">
@@ -11826,7 +11826,7 @@
       </c>
       <c r="B323" t="inlineStr">
         <is>
-          <t>Corylus avellana</t>
+          <t>Corylus Avellana</t>
         </is>
       </c>
       <c r="C323" t="inlineStr">
@@ -11859,7 +11859,7 @@
       </c>
       <c r="B324" t="inlineStr">
         <is>
-          <t>Corylus avellana</t>
+          <t>Corylus Avellana</t>
         </is>
       </c>
       <c r="C324" t="inlineStr">
@@ -11925,7 +11925,7 @@
       </c>
       <c r="B326" t="inlineStr">
         <is>
-          <t>Corylus colurna</t>
+          <t>Corylus Colurna</t>
         </is>
       </c>
       <c r="C326" t="inlineStr">
@@ -11963,7 +11963,7 @@
       </c>
       <c r="B327" t="inlineStr">
         <is>
-          <t>Corylus colurna</t>
+          <t>Corylus Colurna</t>
         </is>
       </c>
       <c r="C327" t="inlineStr">
@@ -12346,7 +12346,7 @@
       </c>
       <c r="B338" t="inlineStr">
         <is>
-          <t>Crataegus monogyna</t>
+          <t>Crataegus Monogyna</t>
         </is>
       </c>
       <c r="C338" t="inlineStr">
@@ -12488,7 +12488,7 @@
       </c>
       <c r="B342" t="inlineStr">
         <is>
-          <t>Crateagus monogyna</t>
+          <t>Crateagus Monogyna</t>
         </is>
       </c>
       <c r="C342" t="inlineStr">
@@ -12526,7 +12526,7 @@
       </c>
       <c r="B343" t="inlineStr">
         <is>
-          <t>Cupressus macrocarpa</t>
+          <t>Cupressus Macrocarpa</t>
         </is>
       </c>
       <c r="C343" t="inlineStr">
@@ -12559,7 +12559,7 @@
       </c>
       <c r="B344" t="inlineStr">
         <is>
-          <t>Cupressus macrocarpa</t>
+          <t>Cupressus Macrocarpa</t>
         </is>
       </c>
       <c r="C344" t="inlineStr">
@@ -12658,7 +12658,7 @@
       </c>
       <c r="B347" t="inlineStr">
         <is>
-          <t>Davidia involucrata</t>
+          <t>Davidia Involucrata</t>
         </is>
       </c>
       <c r="C347" t="inlineStr">
@@ -12691,7 +12691,7 @@
       </c>
       <c r="B348" t="inlineStr">
         <is>
-          <t>Davidia involucrata</t>
+          <t>Davidia Involucrata</t>
         </is>
       </c>
       <c r="C348" t="inlineStr">
@@ -12795,7 +12795,7 @@
       </c>
       <c r="B351" t="inlineStr">
         <is>
-          <t>Eucalyptus dalrympleana</t>
+          <t>Eucalyptus Dalrympleana</t>
         </is>
       </c>
       <c r="C351" t="inlineStr">
@@ -12828,7 +12828,7 @@
       </c>
       <c r="B352" t="inlineStr">
         <is>
-          <t>Eucalyptus gunnii</t>
+          <t>Eucalyptus Gunnii</t>
         </is>
       </c>
       <c r="C352" t="inlineStr">
@@ -12894,7 +12894,7 @@
       </c>
       <c r="B354" t="inlineStr">
         <is>
-          <t>Eucalyptus moorei</t>
+          <t>Eucalyptus Moorei</t>
         </is>
       </c>
       <c r="C354" t="inlineStr">
@@ -12927,7 +12927,7 @@
       </c>
       <c r="B355" t="inlineStr">
         <is>
-          <t>Eucalyptus perriniana</t>
+          <t>Eucalyptus Perriniana</t>
         </is>
       </c>
       <c r="C355" t="inlineStr">
@@ -13409,7 +13409,7 @@
       </c>
       <c r="B369" t="inlineStr">
         <is>
-          <t>Fagus syl.</t>
+          <t>Fagus Syl.</t>
         </is>
       </c>
       <c r="C369" t="inlineStr">
@@ -13480,7 +13480,7 @@
       </c>
       <c r="B371" t="inlineStr">
         <is>
-          <t>Fagus sylvatica</t>
+          <t>Fagus Sylvatica</t>
         </is>
       </c>
       <c r="C371" t="inlineStr">
@@ -13513,7 +13513,7 @@
       </c>
       <c r="B372" t="inlineStr">
         <is>
-          <t>Fagus sylvatica</t>
+          <t>Fagus Sylvatica</t>
         </is>
       </c>
       <c r="C372" t="inlineStr">
@@ -13551,7 +13551,7 @@
       </c>
       <c r="B373" t="inlineStr">
         <is>
-          <t>Fagus sylvatica</t>
+          <t>Fagus Sylvatica</t>
         </is>
       </c>
       <c r="C373" t="inlineStr">
@@ -13589,7 +13589,7 @@
       </c>
       <c r="B374" t="inlineStr">
         <is>
-          <t>Fagus sylvatica</t>
+          <t>Fagus Sylvatica</t>
         </is>
       </c>
       <c r="C374" t="inlineStr">
@@ -13622,7 +13622,7 @@
       </c>
       <c r="B375" t="inlineStr">
         <is>
-          <t>Fargesia robusta</t>
+          <t>Fargesia Robusta</t>
         </is>
       </c>
       <c r="C375" t="inlineStr">
@@ -13721,7 +13721,7 @@
       </c>
       <c r="B378" t="inlineStr">
         <is>
-          <t>Fraxinus angustifolia</t>
+          <t>Fraxinus Angustifolia</t>
         </is>
       </c>
       <c r="D378" t="inlineStr">
@@ -13825,7 +13825,7 @@
       </c>
       <c r="B381" t="inlineStr">
         <is>
-          <t>Gift card</t>
+          <t>Gift Card</t>
         </is>
       </c>
       <c r="D381" t="inlineStr">
@@ -13855,7 +13855,7 @@
       </c>
       <c r="B382" t="inlineStr">
         <is>
-          <t>Ginkgo biloba</t>
+          <t>Ginkgo Biloba</t>
         </is>
       </c>
       <c r="C382" t="inlineStr">
@@ -13888,7 +13888,7 @@
       </c>
       <c r="B383" t="inlineStr">
         <is>
-          <t>Ginkgo biloba</t>
+          <t>Ginkgo Biloba</t>
         </is>
       </c>
       <c r="C383" t="inlineStr">
@@ -13921,7 +13921,7 @@
       </c>
       <c r="B384" t="inlineStr">
         <is>
-          <t>Ginkgo biloba</t>
+          <t>Ginkgo Biloba</t>
         </is>
       </c>
       <c r="C384" t="inlineStr">
@@ -13959,7 +13959,7 @@
       </c>
       <c r="B385" t="inlineStr">
         <is>
-          <t>Ginkgo biloba</t>
+          <t>Ginkgo Biloba</t>
         </is>
       </c>
       <c r="C385" t="inlineStr">
@@ -13992,7 +13992,7 @@
       </c>
       <c r="B386" t="inlineStr">
         <is>
-          <t>Ginkgo biloba</t>
+          <t>Ginkgo Biloba</t>
         </is>
       </c>
       <c r="C386" t="inlineStr">
@@ -14025,7 +14025,7 @@
       </c>
       <c r="B387" t="inlineStr">
         <is>
-          <t>Ginkgo biloba</t>
+          <t>Ginkgo Biloba</t>
         </is>
       </c>
       <c r="C387" t="inlineStr">
@@ -14261,7 +14261,7 @@
       </c>
       <c r="B394" t="inlineStr">
         <is>
-          <t>Halesia carolina</t>
+          <t>Halesia Carolina</t>
         </is>
       </c>
       <c r="C394" t="inlineStr">
@@ -14294,7 +14294,7 @@
       </c>
       <c r="B395" t="inlineStr">
         <is>
-          <t>Halesia carolina</t>
+          <t>Halesia Carolina</t>
         </is>
       </c>
       <c r="C395" t="inlineStr">
@@ -14327,7 +14327,7 @@
       </c>
       <c r="B396" t="inlineStr">
         <is>
-          <t>Halesia carolina</t>
+          <t>Halesia Carolina</t>
         </is>
       </c>
       <c r="C396" t="inlineStr">
@@ -14393,7 +14393,7 @@
       </c>
       <c r="B398" t="inlineStr">
         <is>
-          <t>Heptacodium miconioides</t>
+          <t>Heptacodium Miconioides</t>
         </is>
       </c>
       <c r="C398" t="inlineStr">
@@ -14426,7 +14426,7 @@
       </c>
       <c r="B399" t="inlineStr">
         <is>
-          <t>Heptacodium miconioides</t>
+          <t>Heptacodium Miconioides</t>
         </is>
       </c>
       <c r="C399" t="inlineStr">
@@ -14464,7 +14464,7 @@
       </c>
       <c r="B400" t="inlineStr">
         <is>
-          <t>Heptacodium miconioides</t>
+          <t>Heptacodium Miconioides</t>
         </is>
       </c>
       <c r="C400" t="inlineStr">
@@ -14596,7 +14596,7 @@
       </c>
       <c r="B404" t="inlineStr">
         <is>
-          <t>Ilex aquifolium</t>
+          <t>Ilex Aquifolium</t>
         </is>
       </c>
       <c r="C404" t="inlineStr">
@@ -14629,7 +14629,7 @@
       </c>
       <c r="B405" t="inlineStr">
         <is>
-          <t>Ilex aquifolium</t>
+          <t>Ilex Aquifolium</t>
         </is>
       </c>
       <c r="C405" t="inlineStr">
@@ -14662,7 +14662,7 @@
       </c>
       <c r="B406" t="inlineStr">
         <is>
-          <t>Juglans nigra</t>
+          <t>Juglans Nigra</t>
         </is>
       </c>
       <c r="C406" t="inlineStr">
@@ -14695,7 +14695,7 @@
       </c>
       <c r="B407" t="inlineStr">
         <is>
-          <t>Juglans nigra</t>
+          <t>Juglans Nigra</t>
         </is>
       </c>
       <c r="C407" t="inlineStr">
@@ -14733,7 +14733,7 @@
       </c>
       <c r="B408" t="inlineStr">
         <is>
-          <t>Juglans nigra</t>
+          <t>Juglans Nigra</t>
         </is>
       </c>
       <c r="C408" t="inlineStr">
@@ -14771,7 +14771,7 @@
       </c>
       <c r="B409" t="inlineStr">
         <is>
-          <t>Juglans nigra</t>
+          <t>Juglans Nigra</t>
         </is>
       </c>
       <c r="C409" t="inlineStr">
@@ -14809,7 +14809,7 @@
       </c>
       <c r="B410" t="inlineStr">
         <is>
-          <t>Juglans regia</t>
+          <t>Juglans Regia</t>
         </is>
       </c>
       <c r="C410" t="inlineStr">
@@ -14842,7 +14842,7 @@
       </c>
       <c r="B411" t="inlineStr">
         <is>
-          <t>Juglans regia</t>
+          <t>Juglans Regia</t>
         </is>
       </c>
       <c r="C411" t="inlineStr">
@@ -14875,7 +14875,7 @@
       </c>
       <c r="B412" t="inlineStr">
         <is>
-          <t>Juglans regia</t>
+          <t>Juglans Regia</t>
         </is>
       </c>
       <c r="C412" t="inlineStr">
@@ -15050,7 +15050,7 @@
       </c>
       <c r="B417" t="inlineStr">
         <is>
-          <t>Koelreuteria paniculata</t>
+          <t>Koelreuteria Paniculata</t>
         </is>
       </c>
       <c r="C417" t="inlineStr">
@@ -15083,7 +15083,7 @@
       </c>
       <c r="B418" t="inlineStr">
         <is>
-          <t>Koelreuteria paniculata</t>
+          <t>Koelreuteria Paniculata</t>
         </is>
       </c>
       <c r="C418" t="inlineStr">
@@ -15121,7 +15121,7 @@
       </c>
       <c r="B419" t="inlineStr">
         <is>
-          <t>Koelreuteria paniculata</t>
+          <t>Koelreuteria Paniculata</t>
         </is>
       </c>
       <c r="C419" t="inlineStr">
@@ -15154,7 +15154,7 @@
       </c>
       <c r="B420" t="inlineStr">
         <is>
-          <t>Koelreuteria paniculata</t>
+          <t>Koelreuteria Paniculata</t>
         </is>
       </c>
       <c r="C420" t="inlineStr">
@@ -15225,7 +15225,7 @@
       </c>
       <c r="B422" t="inlineStr">
         <is>
-          <t>Larix decidua</t>
+          <t>Larix Decidua</t>
         </is>
       </c>
       <c r="C422" t="inlineStr">
@@ -15258,7 +15258,7 @@
       </c>
       <c r="B423" t="inlineStr">
         <is>
-          <t>Larix kaempferi</t>
+          <t>Larix Kaempferi</t>
         </is>
       </c>
       <c r="C423" t="inlineStr">
@@ -15291,7 +15291,7 @@
       </c>
       <c r="B424" t="inlineStr">
         <is>
-          <t>Larix kaempferi</t>
+          <t>Larix Kaempferi</t>
         </is>
       </c>
       <c r="C424" t="inlineStr">
@@ -15324,7 +15324,7 @@
       </c>
       <c r="B425" t="inlineStr">
         <is>
-          <t>Larix kaempferi</t>
+          <t>Larix Kaempferi</t>
         </is>
       </c>
       <c r="C425" t="inlineStr">
@@ -15357,7 +15357,7 @@
       </c>
       <c r="B426" t="inlineStr">
         <is>
-          <t>Laurus nobilis</t>
+          <t>Laurus Nobilis</t>
         </is>
       </c>
       <c r="C426" t="inlineStr">
@@ -15390,7 +15390,7 @@
       </c>
       <c r="B427" t="inlineStr">
         <is>
-          <t>Laurus nobilis</t>
+          <t>Laurus Nobilis</t>
         </is>
       </c>
       <c r="C427" t="inlineStr">
@@ -15423,7 +15423,7 @@
       </c>
       <c r="B428" t="inlineStr">
         <is>
-          <t>Liquidambar styraciflua</t>
+          <t>Liquidambar Styraciflua</t>
         </is>
       </c>
       <c r="C428" t="inlineStr">
@@ -15461,7 +15461,7 @@
       </c>
       <c r="B429" t="inlineStr">
         <is>
-          <t>Liquidambar styraciflua</t>
+          <t>Liquidambar Styraciflua</t>
         </is>
       </c>
       <c r="C429" t="inlineStr">
@@ -15499,7 +15499,7 @@
       </c>
       <c r="B430" t="inlineStr">
         <is>
-          <t>Liquidambar styraciflua</t>
+          <t>Liquidambar Styraciflua</t>
         </is>
       </c>
       <c r="C430" t="inlineStr">
@@ -15537,7 +15537,7 @@
       </c>
       <c r="B431" t="inlineStr">
         <is>
-          <t>Liquidambar styraciflua</t>
+          <t>Liquidambar Styraciflua</t>
         </is>
       </c>
       <c r="C431" t="inlineStr">
@@ -15935,7 +15935,7 @@
       </c>
       <c r="B442" t="inlineStr">
         <is>
-          <t>Liriodendron tulipifera</t>
+          <t>Liriodendron Tulipifera</t>
         </is>
       </c>
       <c r="C442" t="inlineStr">
@@ -15968,7 +15968,7 @@
       </c>
       <c r="B443" t="inlineStr">
         <is>
-          <t>Liriodendron tulipifera</t>
+          <t>Liriodendron Tulipifera</t>
         </is>
       </c>
       <c r="C443" t="inlineStr">
@@ -16001,7 +16001,7 @@
       </c>
       <c r="B444" t="inlineStr">
         <is>
-          <t>Liriodendron tulipifera</t>
+          <t>Liriodendron Tulipifera</t>
         </is>
       </c>
       <c r="C444" t="inlineStr">
@@ -16034,7 +16034,7 @@
       </c>
       <c r="B445" t="inlineStr">
         <is>
-          <t>Liriodendron tulipifera</t>
+          <t>Liriodendron Tulipifera</t>
         </is>
       </c>
       <c r="C445" t="inlineStr">
@@ -16072,7 +16072,7 @@
       </c>
       <c r="B446" t="inlineStr">
         <is>
-          <t>Liriodendron tulipifera</t>
+          <t>Liriodendron Tulipifera</t>
         </is>
       </c>
       <c r="C446" t="inlineStr">
@@ -16488,7 +16488,7 @@
       </c>
       <c r="B458" t="inlineStr">
         <is>
-          <t>Magnolia grandiflora</t>
+          <t>Magnolia Grandiflora</t>
         </is>
       </c>
       <c r="C458" t="inlineStr">
@@ -16521,7 +16521,7 @@
       </c>
       <c r="B459" t="inlineStr">
         <is>
-          <t>Magnolia kobus</t>
+          <t>Magnolia Kobus</t>
         </is>
       </c>
       <c r="C459" t="inlineStr">
@@ -16554,7 +16554,7 @@
       </c>
       <c r="B460" t="inlineStr">
         <is>
-          <t>Magnolia stellata</t>
+          <t>Magnolia Stellata</t>
         </is>
       </c>
       <c r="C460" t="inlineStr">
@@ -16587,7 +16587,7 @@
       </c>
       <c r="B461" t="inlineStr">
         <is>
-          <t>Magnolia stellata</t>
+          <t>Magnolia Stellata</t>
         </is>
       </c>
       <c r="C461" t="inlineStr">
@@ -17738,7 +17738,7 @@
       </c>
       <c r="B493" t="inlineStr">
         <is>
-          <t>Malus baccata</t>
+          <t>Malus Baccata</t>
         </is>
       </c>
       <c r="C493" t="inlineStr">
@@ -18502,7 +18502,7 @@
       </c>
       <c r="B516" t="inlineStr">
         <is>
-          <t>Malus domestica</t>
+          <t>Malus Domestica</t>
         </is>
       </c>
       <c r="C516" t="inlineStr">
@@ -18535,7 +18535,7 @@
       </c>
       <c r="B517" t="inlineStr">
         <is>
-          <t>Malus sylvestris</t>
+          <t>Malus Sylvestris</t>
         </is>
       </c>
       <c r="C517" t="inlineStr">
@@ -18568,7 +18568,7 @@
       </c>
       <c r="B518" t="inlineStr">
         <is>
-          <t>Malus trilobata</t>
+          <t>Malus Trilobata</t>
         </is>
       </c>
       <c r="C518" t="inlineStr">
@@ -18601,7 +18601,7 @@
       </c>
       <c r="B519" t="inlineStr">
         <is>
-          <t>Malus trilobata</t>
+          <t>Malus Trilobata</t>
         </is>
       </c>
       <c r="C519" t="inlineStr">
@@ -18639,7 +18639,7 @@
       </c>
       <c r="B520" t="inlineStr">
         <is>
-          <t>Malus trilobata</t>
+          <t>Malus Trilobata</t>
         </is>
       </c>
       <c r="C520" t="inlineStr">
@@ -18677,7 +18677,7 @@
       </c>
       <c r="B521" t="inlineStr">
         <is>
-          <t>Malus trilobata</t>
+          <t>Malus Trilobata</t>
         </is>
       </c>
       <c r="C521" t="inlineStr">
@@ -18715,7 +18715,7 @@
       </c>
       <c r="B522" t="inlineStr">
         <is>
-          <t>Malus trilobata</t>
+          <t>Malus Trilobata</t>
         </is>
       </c>
       <c r="C522" t="inlineStr">
@@ -18753,7 +18753,7 @@
       </c>
       <c r="B523" t="inlineStr">
         <is>
-          <t>Malus trilobata</t>
+          <t>Malus Trilobata</t>
         </is>
       </c>
       <c r="C523" t="inlineStr">
@@ -18791,7 +18791,7 @@
       </c>
       <c r="B524" t="inlineStr">
         <is>
-          <t>Mespilus germanica</t>
+          <t>Mespilus Germanica</t>
         </is>
       </c>
       <c r="C524" t="inlineStr">
@@ -18824,7 +18824,7 @@
       </c>
       <c r="B525" t="inlineStr">
         <is>
-          <t>Metasequoia glytostroboides</t>
+          <t>Metasequoia Glytostroboides</t>
         </is>
       </c>
       <c r="C525" t="inlineStr">
@@ -18862,7 +18862,7 @@
       </c>
       <c r="B526" t="inlineStr">
         <is>
-          <t>Metasequoia glytostroboides</t>
+          <t>Metasequoia Glytostroboides</t>
         </is>
       </c>
       <c r="C526" t="inlineStr">
@@ -18900,7 +18900,7 @@
       </c>
       <c r="B527" t="inlineStr">
         <is>
-          <t>Metasequoia glytostroboides</t>
+          <t>Metasequoia Glytostroboides</t>
         </is>
       </c>
       <c r="C527" t="inlineStr">
@@ -18938,7 +18938,7 @@
       </c>
       <c r="B528" t="inlineStr">
         <is>
-          <t>Metasequoia glytostroboides</t>
+          <t>Metasequoia Glytostroboides</t>
         </is>
       </c>
       <c r="C528" t="inlineStr">
@@ -18976,7 +18976,7 @@
       </c>
       <c r="B529" t="inlineStr">
         <is>
-          <t>Metasequoia glytostroboides</t>
+          <t>Metasequoia Glytostroboides</t>
         </is>
       </c>
       <c r="C529" t="inlineStr">
@@ -19014,7 +19014,7 @@
       </c>
       <c r="B530" t="inlineStr">
         <is>
-          <t>Metasequoia glytostroboides</t>
+          <t>Metasequoia Glytostroboides</t>
         </is>
       </c>
       <c r="C530" t="inlineStr">
@@ -19052,7 +19052,7 @@
       </c>
       <c r="B531" t="inlineStr">
         <is>
-          <t>Morus alba</t>
+          <t>Morus Alba</t>
         </is>
       </c>
       <c r="C531" t="inlineStr">
@@ -19085,7 +19085,7 @@
       </c>
       <c r="B532" t="inlineStr">
         <is>
-          <t>Morus alba</t>
+          <t>Morus Alba</t>
         </is>
       </c>
       <c r="C532" t="inlineStr">
@@ -19118,7 +19118,7 @@
       </c>
       <c r="B533" t="inlineStr">
         <is>
-          <t>Morus alba</t>
+          <t>Morus Alba</t>
         </is>
       </c>
       <c r="C533" t="inlineStr">
@@ -19151,7 +19151,7 @@
       </c>
       <c r="B534" t="inlineStr">
         <is>
-          <t>Morus nigra</t>
+          <t>Morus Nigra</t>
         </is>
       </c>
       <c r="C534" t="inlineStr">
@@ -19184,7 +19184,7 @@
       </c>
       <c r="B535" t="inlineStr">
         <is>
-          <t>Nothofagus antarctica</t>
+          <t>Nothofagus Antarctica</t>
         </is>
       </c>
       <c r="C535" t="inlineStr">
@@ -19217,7 +19217,7 @@
       </c>
       <c r="B536" t="inlineStr">
         <is>
-          <t>Nyssa sylvatica</t>
+          <t>Nyssa Sylvatica</t>
         </is>
       </c>
       <c r="C536" t="inlineStr">
@@ -19250,7 +19250,7 @@
       </c>
       <c r="B537" t="inlineStr">
         <is>
-          <t>Nyssa sylvatica</t>
+          <t>Nyssa Sylvatica</t>
         </is>
       </c>
       <c r="C537" t="inlineStr">
@@ -19283,7 +19283,7 @@
       </c>
       <c r="B538" t="inlineStr">
         <is>
-          <t>Nyssa sylvatica</t>
+          <t>Nyssa Sylvatica</t>
         </is>
       </c>
       <c r="C538" t="inlineStr">
@@ -19316,7 +19316,7 @@
       </c>
       <c r="B539" t="inlineStr">
         <is>
-          <t>Ostrya carpinifolia</t>
+          <t>Ostrya Carpinifolia</t>
         </is>
       </c>
       <c r="C539" t="inlineStr">
@@ -19349,7 +19349,7 @@
       </c>
       <c r="B540" t="inlineStr">
         <is>
-          <t>Ostrya carpinifolia</t>
+          <t>Ostrya Carpinifolia</t>
         </is>
       </c>
       <c r="C540" t="inlineStr">
@@ -19387,7 +19387,7 @@
       </c>
       <c r="B541" t="inlineStr">
         <is>
-          <t>Ostrya carpinifolia</t>
+          <t>Ostrya Carpinifolia</t>
         </is>
       </c>
       <c r="C541" t="inlineStr">
@@ -19425,7 +19425,7 @@
       </c>
       <c r="B542" t="inlineStr">
         <is>
-          <t>Parrotia persica</t>
+          <t>Parrotia Persica</t>
         </is>
       </c>
       <c r="C542" t="inlineStr">
@@ -19463,7 +19463,7 @@
       </c>
       <c r="B543" t="inlineStr">
         <is>
-          <t>Parrotia persica</t>
+          <t>Parrotia Persica</t>
         </is>
       </c>
       <c r="C543" t="inlineStr">
@@ -19704,7 +19704,7 @@
       </c>
       <c r="B550" t="inlineStr">
         <is>
-          <t>Paulownia tomentosa</t>
+          <t>Paulownia Tomentosa</t>
         </is>
       </c>
       <c r="C550" t="inlineStr">
@@ -19742,7 +19742,7 @@
       </c>
       <c r="B551" t="inlineStr">
         <is>
-          <t>Paulownia tomentosa</t>
+          <t>Paulownia Tomentosa</t>
         </is>
       </c>
       <c r="C551" t="inlineStr">
@@ -19775,7 +19775,7 @@
       </c>
       <c r="B552" t="inlineStr">
         <is>
-          <t>Phellodendron amurense</t>
+          <t>Phellodendron Amurense</t>
         </is>
       </c>
       <c r="C552" t="inlineStr">
@@ -19808,7 +19808,7 @@
       </c>
       <c r="B553" t="inlineStr">
         <is>
-          <t>Picea abies</t>
+          <t>Picea Abies</t>
         </is>
       </c>
       <c r="C553" t="inlineStr">
@@ -19841,7 +19841,7 @@
       </c>
       <c r="B554" t="inlineStr">
         <is>
-          <t>Picea abies</t>
+          <t>Picea Abies</t>
         </is>
       </c>
       <c r="C554" t="inlineStr">
@@ -19874,7 +19874,7 @@
       </c>
       <c r="B555" t="inlineStr">
         <is>
-          <t>Picea abies</t>
+          <t>Picea Abies</t>
         </is>
       </c>
       <c r="C555" t="inlineStr">
@@ -19940,7 +19940,7 @@
       </c>
       <c r="B557" t="inlineStr">
         <is>
-          <t>Picea omorika</t>
+          <t>Picea Omorika</t>
         </is>
       </c>
       <c r="C557" t="inlineStr">
@@ -19973,7 +19973,7 @@
       </c>
       <c r="B558" t="inlineStr">
         <is>
-          <t>Picea pungens</t>
+          <t>Picea Pungens</t>
         </is>
       </c>
       <c r="C558" t="inlineStr">
@@ -20006,7 +20006,7 @@
       </c>
       <c r="B559" t="inlineStr">
         <is>
-          <t>Picea sitchensis</t>
+          <t>Picea Sitchensis</t>
         </is>
       </c>
       <c r="C559" t="inlineStr">
@@ -20039,7 +20039,7 @@
       </c>
       <c r="B560" t="inlineStr">
         <is>
-          <t>Pinus armandii</t>
+          <t>Pinus Armandii</t>
         </is>
       </c>
       <c r="C560" t="inlineStr">
@@ -20072,7 +20072,7 @@
       </c>
       <c r="B561" t="inlineStr">
         <is>
-          <t>Pinus contorta</t>
+          <t>Pinus Contorta</t>
         </is>
       </c>
       <c r="C561" t="inlineStr">
@@ -20105,7 +20105,7 @@
       </c>
       <c r="B562" t="inlineStr">
         <is>
-          <t>Pinus halepensis</t>
+          <t>Pinus Halepensis</t>
         </is>
       </c>
       <c r="C562" t="inlineStr">
@@ -20138,7 +20138,7 @@
       </c>
       <c r="B563" t="inlineStr">
         <is>
-          <t>Pinus mugo</t>
+          <t>Pinus Mugo</t>
         </is>
       </c>
       <c r="C563" t="inlineStr">
@@ -20171,7 +20171,7 @@
       </c>
       <c r="B564" t="inlineStr">
         <is>
-          <t>Pinus mugo</t>
+          <t>Pinus Mugo</t>
         </is>
       </c>
       <c r="C564" t="inlineStr">
@@ -20204,7 +20204,7 @@
       </c>
       <c r="B565" t="inlineStr">
         <is>
-          <t>Pinus mugo</t>
+          <t>Pinus Mugo</t>
         </is>
       </c>
       <c r="C565" t="inlineStr">
@@ -20237,7 +20237,7 @@
       </c>
       <c r="B566" t="inlineStr">
         <is>
-          <t>Pinus nigra</t>
+          <t>Pinus Nigra</t>
         </is>
       </c>
       <c r="C566" t="inlineStr">
@@ -20270,7 +20270,7 @@
       </c>
       <c r="B567" t="inlineStr">
         <is>
-          <t>Pinus nigra</t>
+          <t>Pinus Nigra</t>
         </is>
       </c>
       <c r="C567" t="inlineStr">
@@ -20303,7 +20303,7 @@
       </c>
       <c r="B568" t="inlineStr">
         <is>
-          <t>Pinus nigra</t>
+          <t>Pinus Nigra</t>
         </is>
       </c>
       <c r="C568" t="inlineStr">
@@ -20336,7 +20336,7 @@
       </c>
       <c r="B569" t="inlineStr">
         <is>
-          <t>Pinus nigra</t>
+          <t>Pinus Nigra</t>
         </is>
       </c>
       <c r="C569" t="inlineStr">
@@ -20374,7 +20374,7 @@
       </c>
       <c r="B570" t="inlineStr">
         <is>
-          <t>Pinus pinaster</t>
+          <t>Pinus Pinaster</t>
         </is>
       </c>
       <c r="C570" t="inlineStr">
@@ -20412,7 +20412,7 @@
       </c>
       <c r="B571" t="inlineStr">
         <is>
-          <t>Pinus pinaster</t>
+          <t>Pinus Pinaster</t>
         </is>
       </c>
       <c r="C571" t="inlineStr">
@@ -20445,7 +20445,7 @@
       </c>
       <c r="B572" t="inlineStr">
         <is>
-          <t>Pinus pinea</t>
+          <t>Pinus Pinea</t>
         </is>
       </c>
       <c r="C572" t="inlineStr">
@@ -20478,7 +20478,7 @@
       </c>
       <c r="B573" t="inlineStr">
         <is>
-          <t>Pinus ponderosa</t>
+          <t>Pinus Ponderosa</t>
         </is>
       </c>
       <c r="C573" t="inlineStr">
@@ -20511,7 +20511,7 @@
       </c>
       <c r="B574" t="inlineStr">
         <is>
-          <t>Pinus strobus</t>
+          <t>Pinus Strobus</t>
         </is>
       </c>
       <c r="C574" t="inlineStr">
@@ -20544,7 +20544,7 @@
       </c>
       <c r="B575" t="inlineStr">
         <is>
-          <t>Pinus strobus</t>
+          <t>Pinus Strobus</t>
         </is>
       </c>
       <c r="C575" t="inlineStr">
@@ -20577,7 +20577,7 @@
       </c>
       <c r="B576" t="inlineStr">
         <is>
-          <t>Pinus strobus</t>
+          <t>Pinus Strobus</t>
         </is>
       </c>
       <c r="C576" t="inlineStr">
@@ -20610,7 +20610,7 @@
       </c>
       <c r="B577" t="inlineStr">
         <is>
-          <t>Pinus sylvestris</t>
+          <t>Pinus Sylvestris</t>
         </is>
       </c>
       <c r="C577" t="inlineStr">
@@ -20643,7 +20643,7 @@
       </c>
       <c r="B578" t="inlineStr">
         <is>
-          <t>Pinus sylvestris</t>
+          <t>Pinus Sylvestris</t>
         </is>
       </c>
       <c r="C578" t="inlineStr">
@@ -20676,7 +20676,7 @@
       </c>
       <c r="B579" t="inlineStr">
         <is>
-          <t>Pinus tabuliformis</t>
+          <t>Pinus Tabuliformis</t>
         </is>
       </c>
       <c r="C579" t="inlineStr">
@@ -20709,7 +20709,7 @@
       </c>
       <c r="B580" t="inlineStr">
         <is>
-          <t>Pinus tabuliformis</t>
+          <t>Pinus Tabuliformis</t>
         </is>
       </c>
       <c r="C580" t="inlineStr">
@@ -20742,7 +20742,7 @@
       </c>
       <c r="B581" t="inlineStr">
         <is>
-          <t>Pinus wallichiana</t>
+          <t>Pinus Wallichiana</t>
         </is>
       </c>
       <c r="C581" t="inlineStr">
@@ -20775,7 +20775,7 @@
       </c>
       <c r="B582" t="inlineStr">
         <is>
-          <t>Pinus wallichiana</t>
+          <t>Pinus Wallichiana</t>
         </is>
       </c>
       <c r="C582" t="inlineStr">
@@ -20808,7 +20808,7 @@
       </c>
       <c r="B583" t="inlineStr">
         <is>
-          <t>Platanus orientalis</t>
+          <t>Platanus Orientalis</t>
         </is>
       </c>
       <c r="C583" t="inlineStr">
@@ -20841,7 +20841,7 @@
       </c>
       <c r="B584" t="inlineStr">
         <is>
-          <t>Platanus orientalis</t>
+          <t>Platanus Orientalis</t>
         </is>
       </c>
       <c r="C584" t="inlineStr">
@@ -20874,7 +20874,7 @@
       </c>
       <c r="B585" t="inlineStr">
         <is>
-          <t>Platanus orientalis</t>
+          <t>Platanus Orientalis</t>
         </is>
       </c>
       <c r="C585" t="inlineStr">
@@ -20912,7 +20912,7 @@
       </c>
       <c r="B586" t="inlineStr">
         <is>
-          <t>Platanus orientalis</t>
+          <t>Platanus Orientalis</t>
         </is>
       </c>
       <c r="C586" t="inlineStr">
@@ -20950,7 +20950,7 @@
       </c>
       <c r="B587" t="inlineStr">
         <is>
-          <t>Platanus orientalis</t>
+          <t>Platanus Orientalis</t>
         </is>
       </c>
       <c r="C587" t="inlineStr">
@@ -20988,7 +20988,7 @@
       </c>
       <c r="B588" t="inlineStr">
         <is>
-          <t>Platanus orientalis</t>
+          <t>Platanus Orientalis</t>
         </is>
       </c>
       <c r="C588" t="inlineStr">
@@ -21026,7 +21026,7 @@
       </c>
       <c r="B589" t="inlineStr">
         <is>
-          <t>Platanus x</t>
+          <t>Platanus X</t>
         </is>
       </c>
       <c r="C589" t="inlineStr">
@@ -21059,7 +21059,7 @@
       </c>
       <c r="B590" t="inlineStr">
         <is>
-          <t>Platanus x</t>
+          <t>Platanus X</t>
         </is>
       </c>
       <c r="C590" t="inlineStr">
@@ -21097,7 +21097,7 @@
       </c>
       <c r="B591" t="inlineStr">
         <is>
-          <t>Platanus x</t>
+          <t>Platanus X</t>
         </is>
       </c>
       <c r="C591" t="inlineStr">
@@ -21135,7 +21135,7 @@
       </c>
       <c r="B592" t="inlineStr">
         <is>
-          <t>Platanus x</t>
+          <t>Platanus X</t>
         </is>
       </c>
       <c r="C592" t="inlineStr">
@@ -21173,7 +21173,7 @@
       </c>
       <c r="B593" t="inlineStr">
         <is>
-          <t>Platanus x</t>
+          <t>Platanus X</t>
         </is>
       </c>
       <c r="C593" t="inlineStr">
@@ -21211,7 +21211,7 @@
       </c>
       <c r="B594" t="inlineStr">
         <is>
-          <t>Platanus x</t>
+          <t>Platanus X</t>
         </is>
       </c>
       <c r="C594" t="inlineStr">
@@ -21249,7 +21249,7 @@
       </c>
       <c r="B595" t="inlineStr">
         <is>
-          <t>Populus alba</t>
+          <t>Populus Alba</t>
         </is>
       </c>
       <c r="C595" t="inlineStr">
@@ -21282,7 +21282,7 @@
       </c>
       <c r="B596" t="inlineStr">
         <is>
-          <t>Populus tremula</t>
+          <t>Populus Tremula</t>
         </is>
       </c>
       <c r="C596" t="inlineStr">
@@ -21320,7 +21320,7 @@
       </c>
       <c r="B597" t="inlineStr">
         <is>
-          <t>Populus tremula</t>
+          <t>Populus Tremula</t>
         </is>
       </c>
       <c r="C597" t="inlineStr">
@@ -21353,7 +21353,7 @@
       </c>
       <c r="B598" t="inlineStr">
         <is>
-          <t>Populus tremula</t>
+          <t>Populus Tremula</t>
         </is>
       </c>
       <c r="C598" t="inlineStr">
@@ -21391,7 +21391,7 @@
       </c>
       <c r="B599" t="inlineStr">
         <is>
-          <t>Populus tremula</t>
+          <t>Populus Tremula</t>
         </is>
       </c>
       <c r="C599" t="inlineStr">
@@ -21429,7 +21429,7 @@
       </c>
       <c r="B600" t="inlineStr">
         <is>
-          <t>Populus tremula</t>
+          <t>Populus Tremula</t>
         </is>
       </c>
       <c r="C600" t="inlineStr">
@@ -21467,7 +21467,7 @@
       </c>
       <c r="B601" t="inlineStr">
         <is>
-          <t>Populus tremula</t>
+          <t>Populus Tremula</t>
         </is>
       </c>
       <c r="C601" t="inlineStr">
@@ -21959,7 +21959,7 @@
       </c>
       <c r="B615" t="inlineStr">
         <is>
-          <t>Prunus avium</t>
+          <t>Prunus Avium</t>
         </is>
       </c>
       <c r="C615" t="inlineStr">
@@ -21992,7 +21992,7 @@
       </c>
       <c r="B616" t="inlineStr">
         <is>
-          <t>Prunus avium</t>
+          <t>Prunus Avium</t>
         </is>
       </c>
       <c r="C616" t="inlineStr">
@@ -22626,7 +22626,7 @@
       </c>
       <c r="B634" t="inlineStr">
         <is>
-          <t>Prunus l.</t>
+          <t>Prunus L.</t>
         </is>
       </c>
       <c r="C634" t="inlineStr">
@@ -22664,7 +22664,7 @@
       </c>
       <c r="B635" t="inlineStr">
         <is>
-          <t>Prunus l.</t>
+          <t>Prunus L.</t>
         </is>
       </c>
       <c r="C635" t="inlineStr">
@@ -22882,7 +22882,7 @@
       </c>
       <c r="B641" t="inlineStr">
         <is>
-          <t>Prunus padus</t>
+          <t>Prunus Padus</t>
         </is>
       </c>
       <c r="C641" t="inlineStr">
@@ -23067,7 +23067,7 @@
       </c>
       <c r="B646" t="inlineStr">
         <is>
-          <t>Prunus serrulata</t>
+          <t>Prunus Serrulata</t>
         </is>
       </c>
       <c r="C646" t="inlineStr">
@@ -23100,7 +23100,7 @@
       </c>
       <c r="B647" t="inlineStr">
         <is>
-          <t>Prunus serrulata</t>
+          <t>Prunus Serrulata</t>
         </is>
       </c>
       <c r="C647" t="inlineStr">
@@ -23133,7 +23133,7 @@
       </c>
       <c r="B648" t="inlineStr">
         <is>
-          <t>Prunus serrulata</t>
+          <t>Prunus Serrulata</t>
         </is>
       </c>
       <c r="C648" t="inlineStr">
@@ -23171,7 +23171,7 @@
       </c>
       <c r="B649" t="inlineStr">
         <is>
-          <t>Prunus serrulata</t>
+          <t>Prunus Serrulata</t>
         </is>
       </c>
       <c r="C649" t="inlineStr">
@@ -23209,7 +23209,7 @@
       </c>
       <c r="B650" t="inlineStr">
         <is>
-          <t>Prunus serrulata</t>
+          <t>Prunus Serrulata</t>
         </is>
       </c>
       <c r="C650" t="inlineStr">
@@ -23247,7 +23247,7 @@
       </c>
       <c r="B651" t="inlineStr">
         <is>
-          <t>Prunus serrulata</t>
+          <t>Prunus Serrulata</t>
         </is>
       </c>
       <c r="C651" t="inlineStr">
@@ -23318,7 +23318,7 @@
       </c>
       <c r="B653" t="inlineStr">
         <is>
-          <t>Prunus serrulata</t>
+          <t>Prunus Serrulata</t>
         </is>
       </c>
       <c r="C653" t="inlineStr">
@@ -23465,7 +23465,7 @@
       </c>
       <c r="B657" t="inlineStr">
         <is>
-          <t>Pterocarya fraxinifolia</t>
+          <t>Pterocarya Fraxinifolia</t>
         </is>
       </c>
       <c r="C657" t="inlineStr">
@@ -23503,7 +23503,7 @@
       </c>
       <c r="B658" t="inlineStr">
         <is>
-          <t>Pterocarya fraxinifolia</t>
+          <t>Pterocarya Fraxinifolia</t>
         </is>
       </c>
       <c r="C658" t="inlineStr">
@@ -23536,7 +23536,7 @@
       </c>
       <c r="B659" t="inlineStr">
         <is>
-          <t>Pterocarya fraxinifolia</t>
+          <t>Pterocarya Fraxinifolia</t>
         </is>
       </c>
       <c r="C659" t="inlineStr">
@@ -23574,7 +23574,7 @@
       </c>
       <c r="B660" t="inlineStr">
         <is>
-          <t>Pyrus calleryana</t>
+          <t>Pyrus Calleryana</t>
         </is>
       </c>
       <c r="C660" t="inlineStr">
@@ -23934,7 +23934,7 @@
       </c>
       <c r="B670" t="inlineStr">
         <is>
-          <t>Pyrus communis</t>
+          <t>Pyrus Communis</t>
         </is>
       </c>
       <c r="C670" t="inlineStr">
@@ -23967,7 +23967,7 @@
       </c>
       <c r="B671" t="inlineStr">
         <is>
-          <t>Pyrus communis</t>
+          <t>Pyrus Communis</t>
         </is>
       </c>
       <c r="C671" t="inlineStr">
@@ -24170,7 +24170,7 @@
       </c>
       <c r="B677" t="inlineStr">
         <is>
-          <t>Pyrus salicifolia</t>
+          <t>Pyrus Salicifolia</t>
         </is>
       </c>
       <c r="C677" t="inlineStr">
@@ -24208,7 +24208,7 @@
       </c>
       <c r="B678" t="inlineStr">
         <is>
-          <t>Quercus acutissima</t>
+          <t>Quercus Acutissima</t>
         </is>
       </c>
       <c r="C678" t="inlineStr">
@@ -24246,7 +24246,7 @@
       </c>
       <c r="B679" t="inlineStr">
         <is>
-          <t>Quercus acutissima</t>
+          <t>Quercus Acutissima</t>
         </is>
       </c>
       <c r="C679" t="inlineStr">
@@ -24284,7 +24284,7 @@
       </c>
       <c r="B680" t="inlineStr">
         <is>
-          <t>Quercus acutissima</t>
+          <t>Quercus Acutissima</t>
         </is>
       </c>
       <c r="C680" t="inlineStr">
@@ -24322,7 +24322,7 @@
       </c>
       <c r="B681" t="inlineStr">
         <is>
-          <t>Quercus acutissima</t>
+          <t>Quercus Acutissima</t>
         </is>
       </c>
       <c r="C681" t="inlineStr">
@@ -24360,7 +24360,7 @@
       </c>
       <c r="B682" t="inlineStr">
         <is>
-          <t>Quercus acutissima</t>
+          <t>Quercus Acutissima</t>
         </is>
       </c>
       <c r="C682" t="inlineStr">
@@ -24393,7 +24393,7 @@
       </c>
       <c r="B683" t="inlineStr">
         <is>
-          <t>Quercus bicolor</t>
+          <t>Quercus Bicolor</t>
         </is>
       </c>
       <c r="C683" t="inlineStr">
@@ -24426,7 +24426,7 @@
       </c>
       <c r="B684" t="inlineStr">
         <is>
-          <t>Quercus buckleyi</t>
+          <t>Quercus Buckleyi</t>
         </is>
       </c>
       <c r="C684" t="inlineStr">
@@ -24568,7 +24568,7 @@
       </c>
       <c r="B688" t="inlineStr">
         <is>
-          <t>Quercus cerris</t>
+          <t>Quercus Cerris</t>
         </is>
       </c>
       <c r="C688" t="inlineStr">
@@ -24601,7 +24601,7 @@
       </c>
       <c r="B689" t="inlineStr">
         <is>
-          <t>Quercus cerris</t>
+          <t>Quercus Cerris</t>
         </is>
       </c>
       <c r="C689" t="inlineStr">
@@ -24639,7 +24639,7 @@
       </c>
       <c r="B690" t="inlineStr">
         <is>
-          <t>Quercus cerris</t>
+          <t>Quercus Cerris</t>
         </is>
       </c>
       <c r="C690" t="inlineStr">
@@ -24677,7 +24677,7 @@
       </c>
       <c r="B691" t="inlineStr">
         <is>
-          <t>Quercus cerris</t>
+          <t>Quercus Cerris</t>
         </is>
       </c>
       <c r="C691" t="inlineStr">
@@ -24715,7 +24715,7 @@
       </c>
       <c r="B692" t="inlineStr">
         <is>
-          <t>Quercus cerris</t>
+          <t>Quercus Cerris</t>
         </is>
       </c>
       <c r="C692" t="inlineStr">
@@ -24753,7 +24753,7 @@
       </c>
       <c r="B693" t="inlineStr">
         <is>
-          <t>Quercus cerris</t>
+          <t>Quercus Cerris</t>
         </is>
       </c>
       <c r="C693" t="inlineStr">
@@ -24791,7 +24791,7 @@
       </c>
       <c r="B694" t="inlineStr">
         <is>
-          <t>Quercus coccinea</t>
+          <t>Quercus Coccinea</t>
         </is>
       </c>
       <c r="C694" t="inlineStr">
@@ -24857,7 +24857,7 @@
       </c>
       <c r="B696" t="inlineStr">
         <is>
-          <t>Quercus ilex</t>
+          <t>Quercus Ilex</t>
         </is>
       </c>
       <c r="C696" t="inlineStr">
@@ -24890,7 +24890,7 @@
       </c>
       <c r="B697" t="inlineStr">
         <is>
-          <t>Quercus ilex</t>
+          <t>Quercus Ilex</t>
         </is>
       </c>
       <c r="C697" t="inlineStr">
@@ -24928,7 +24928,7 @@
       </c>
       <c r="B698" t="inlineStr">
         <is>
-          <t>Quercus ilex</t>
+          <t>Quercus Ilex</t>
         </is>
       </c>
       <c r="C698" t="inlineStr">
@@ -24966,7 +24966,7 @@
       </c>
       <c r="B699" t="inlineStr">
         <is>
-          <t>Quercus ilex</t>
+          <t>Quercus Ilex</t>
         </is>
       </c>
       <c r="C699" t="inlineStr">
@@ -24999,7 +24999,7 @@
       </c>
       <c r="B700" t="inlineStr">
         <is>
-          <t>Quercus imbricaria</t>
+          <t>Quercus Imbricaria</t>
         </is>
       </c>
       <c r="C700" t="inlineStr">
@@ -25032,7 +25032,7 @@
       </c>
       <c r="B701" t="inlineStr">
         <is>
-          <t>Quercus imbricaria</t>
+          <t>Quercus Imbricaria</t>
         </is>
       </c>
       <c r="C701" t="inlineStr">
@@ -25070,7 +25070,7 @@
       </c>
       <c r="B702" t="inlineStr">
         <is>
-          <t>Quercus macrocarpa</t>
+          <t>Quercus Macrocarpa</t>
         </is>
       </c>
       <c r="C702" t="inlineStr">
@@ -25103,7 +25103,7 @@
       </c>
       <c r="B703" t="inlineStr">
         <is>
-          <t>Quercus myrsinifolia</t>
+          <t>Quercus Myrsinifolia</t>
         </is>
       </c>
       <c r="C703" t="inlineStr">
@@ -25136,7 +25136,7 @@
       </c>
       <c r="B704" t="inlineStr">
         <is>
-          <t>Quercus myrsinifolia</t>
+          <t>Quercus Myrsinifolia</t>
         </is>
       </c>
       <c r="C704" t="inlineStr">
@@ -25169,7 +25169,7 @@
       </c>
       <c r="B705" t="inlineStr">
         <is>
-          <t>Quercus nigra</t>
+          <t>Quercus Nigra</t>
         </is>
       </c>
       <c r="C705" t="inlineStr">
@@ -25202,7 +25202,7 @@
       </c>
       <c r="B706" t="inlineStr">
         <is>
-          <t>Quercus nigra</t>
+          <t>Quercus Nigra</t>
         </is>
       </c>
       <c r="C706" t="inlineStr">
@@ -25240,7 +25240,7 @@
       </c>
       <c r="B707" t="inlineStr">
         <is>
-          <t>Quercus nigra</t>
+          <t>Quercus Nigra</t>
         </is>
       </c>
       <c r="C707" t="inlineStr">
@@ -25278,7 +25278,7 @@
       </c>
       <c r="B708" t="inlineStr">
         <is>
-          <t>Quercus nigra</t>
+          <t>Quercus Nigra</t>
         </is>
       </c>
       <c r="C708" t="inlineStr">
@@ -25311,7 +25311,7 @@
       </c>
       <c r="B709" t="inlineStr">
         <is>
-          <t>Quercus palustris</t>
+          <t>Quercus Palustris</t>
         </is>
       </c>
       <c r="C709" t="inlineStr">
@@ -25344,7 +25344,7 @@
       </c>
       <c r="B710" t="inlineStr">
         <is>
-          <t>Quercus palustris</t>
+          <t>Quercus Palustris</t>
         </is>
       </c>
       <c r="C710" t="inlineStr">
@@ -25377,7 +25377,7 @@
       </c>
       <c r="B711" t="inlineStr">
         <is>
-          <t>Quercus palustris</t>
+          <t>Quercus Palustris</t>
         </is>
       </c>
       <c r="C711" t="inlineStr">
@@ -25415,7 +25415,7 @@
       </c>
       <c r="B712" t="inlineStr">
         <is>
-          <t>Quercus palustris</t>
+          <t>Quercus Palustris</t>
         </is>
       </c>
       <c r="C712" t="inlineStr">
@@ -25453,7 +25453,7 @@
       </c>
       <c r="B713" t="inlineStr">
         <is>
-          <t>Quercus palustris</t>
+          <t>Quercus Palustris</t>
         </is>
       </c>
       <c r="C713" t="inlineStr">
@@ -25628,7 +25628,7 @@
       </c>
       <c r="B718" t="inlineStr">
         <is>
-          <t>Quercus petraea</t>
+          <t>Quercus Petraea</t>
         </is>
       </c>
       <c r="C718" t="inlineStr">
@@ -25661,7 +25661,7 @@
       </c>
       <c r="B719" t="inlineStr">
         <is>
-          <t>Quercus petraea</t>
+          <t>Quercus Petraea</t>
         </is>
       </c>
       <c r="C719" t="inlineStr">
@@ -25699,7 +25699,7 @@
       </c>
       <c r="B720" t="inlineStr">
         <is>
-          <t>Quercus petraea</t>
+          <t>Quercus Petraea</t>
         </is>
       </c>
       <c r="C720" t="inlineStr">
@@ -25732,7 +25732,7 @@
       </c>
       <c r="B721" t="inlineStr">
         <is>
-          <t>Quercus phellos</t>
+          <t>Quercus Phellos</t>
         </is>
       </c>
       <c r="C721" t="inlineStr">
@@ -25770,7 +25770,7 @@
       </c>
       <c r="B722" t="inlineStr">
         <is>
-          <t>Quercus phillyreoides</t>
+          <t>Quercus Phillyreoides</t>
         </is>
       </c>
       <c r="C722" t="inlineStr">
@@ -25803,7 +25803,7 @@
       </c>
       <c r="B723" t="inlineStr">
         <is>
-          <t>Quercus phillyreoides</t>
+          <t>Quercus Phillyreoides</t>
         </is>
       </c>
       <c r="C723" t="inlineStr">
@@ -25836,7 +25836,7 @@
       </c>
       <c r="B724" t="inlineStr">
         <is>
-          <t>Quercus phillyreoides</t>
+          <t>Quercus Phillyreoides</t>
         </is>
       </c>
       <c r="C724" t="inlineStr">
@@ -25869,7 +25869,7 @@
       </c>
       <c r="B725" t="inlineStr">
         <is>
-          <t>Quercus pubescens</t>
+          <t>Quercus Pubescens</t>
         </is>
       </c>
       <c r="C725" t="inlineStr">
@@ -25902,7 +25902,7 @@
       </c>
       <c r="B726" t="inlineStr">
         <is>
-          <t>Quercus pubescens</t>
+          <t>Quercus Pubescens</t>
         </is>
       </c>
       <c r="C726" t="inlineStr">
@@ -25940,7 +25940,7 @@
       </c>
       <c r="B727" t="inlineStr">
         <is>
-          <t>Quercus pubescens</t>
+          <t>Quercus Pubescens</t>
         </is>
       </c>
       <c r="C727" t="inlineStr">
@@ -25978,7 +25978,7 @@
       </c>
       <c r="B728" t="inlineStr">
         <is>
-          <t>Quercus pubescens</t>
+          <t>Quercus Pubescens</t>
         </is>
       </c>
       <c r="C728" t="inlineStr">
@@ -26016,7 +26016,7 @@
       </c>
       <c r="B729" t="inlineStr">
         <is>
-          <t>Quercus pyrenaica</t>
+          <t>Quercus Pyrenaica</t>
         </is>
       </c>
       <c r="C729" t="inlineStr">
@@ -26054,7 +26054,7 @@
       </c>
       <c r="B730" t="inlineStr">
         <is>
-          <t>Quercus robur</t>
+          <t>Quercus Robur</t>
         </is>
       </c>
       <c r="C730" t="inlineStr">
@@ -26087,7 +26087,7 @@
       </c>
       <c r="B731" t="inlineStr">
         <is>
-          <t>Quercus robur</t>
+          <t>Quercus Robur</t>
         </is>
       </c>
       <c r="C731" t="inlineStr">
@@ -26125,7 +26125,7 @@
       </c>
       <c r="B732" t="inlineStr">
         <is>
-          <t>Quercus robur</t>
+          <t>Quercus Robur</t>
         </is>
       </c>
       <c r="C732" t="inlineStr">
@@ -26158,7 +26158,7 @@
       </c>
       <c r="B733" t="inlineStr">
         <is>
-          <t>Quercus robur</t>
+          <t>Quercus Robur</t>
         </is>
       </c>
       <c r="C733" t="inlineStr">
@@ -26196,7 +26196,7 @@
       </c>
       <c r="B734" t="inlineStr">
         <is>
-          <t>Quercus robur</t>
+          <t>Quercus Robur</t>
         </is>
       </c>
       <c r="C734" t="inlineStr">
@@ -26229,7 +26229,7 @@
       </c>
       <c r="B735" t="inlineStr">
         <is>
-          <t>Quercus robur</t>
+          <t>Quercus Robur</t>
         </is>
       </c>
       <c r="C735" t="inlineStr">
@@ -26267,7 +26267,7 @@
       </c>
       <c r="B736" t="inlineStr">
         <is>
-          <t>Quercus robur</t>
+          <t>Quercus Robur</t>
         </is>
       </c>
       <c r="C736" t="inlineStr">
@@ -26305,7 +26305,7 @@
       </c>
       <c r="B737" t="inlineStr">
         <is>
-          <t>Quercus robur</t>
+          <t>Quercus Robur</t>
         </is>
       </c>
       <c r="C737" t="inlineStr">
@@ -26343,7 +26343,7 @@
       </c>
       <c r="B738" t="inlineStr">
         <is>
-          <t>Quercus robur</t>
+          <t>Quercus Robur</t>
         </is>
       </c>
       <c r="C738" t="inlineStr">
@@ -26452,7 +26452,7 @@
       </c>
       <c r="B741" t="inlineStr">
         <is>
-          <t>Quercus rubra</t>
+          <t>Quercus Rubra</t>
         </is>
       </c>
       <c r="C741" t="inlineStr">
@@ -26485,7 +26485,7 @@
       </c>
       <c r="B742" t="inlineStr">
         <is>
-          <t>Quercus rubra</t>
+          <t>Quercus Rubra</t>
         </is>
       </c>
       <c r="C742" t="inlineStr">
@@ -26518,7 +26518,7 @@
       </c>
       <c r="B743" t="inlineStr">
         <is>
-          <t>Quercus rubra</t>
+          <t>Quercus Rubra</t>
         </is>
       </c>
       <c r="C743" t="inlineStr">
@@ -26556,7 +26556,7 @@
       </c>
       <c r="B744" t="inlineStr">
         <is>
-          <t>Quercus rubra</t>
+          <t>Quercus Rubra</t>
         </is>
       </c>
       <c r="C744" t="inlineStr">
@@ -26594,7 +26594,7 @@
       </c>
       <c r="B745" t="inlineStr">
         <is>
-          <t>Quercus rubra</t>
+          <t>Quercus Rubra</t>
         </is>
       </c>
       <c r="C745" t="inlineStr">
@@ -26627,7 +26627,7 @@
       </c>
       <c r="B746" t="inlineStr">
         <is>
-          <t>Quercus suber</t>
+          <t>Quercus Suber</t>
         </is>
       </c>
       <c r="C746" t="inlineStr">
@@ -26660,7 +26660,7 @@
       </c>
       <c r="B747" t="inlineStr">
         <is>
-          <t>Quercus texana</t>
+          <t>Quercus Texana</t>
         </is>
       </c>
       <c r="C747" t="inlineStr">
@@ -26769,7 +26769,7 @@
       </c>
       <c r="B750" t="inlineStr">
         <is>
-          <t>Rhus typhina</t>
+          <t>Rhus Typhina</t>
         </is>
       </c>
       <c r="C750" t="inlineStr">
@@ -26802,7 +26802,7 @@
       </c>
       <c r="B751" t="inlineStr">
         <is>
-          <t>Rhus typhina</t>
+          <t>Rhus Typhina</t>
         </is>
       </c>
       <c r="C751" t="inlineStr">
@@ -26835,7 +26835,7 @@
       </c>
       <c r="B752" t="inlineStr">
         <is>
-          <t>Rhus typhina</t>
+          <t>Rhus Typhina</t>
         </is>
       </c>
       <c r="C752" t="inlineStr">
@@ -26868,7 +26868,7 @@
       </c>
       <c r="B753" t="inlineStr">
         <is>
-          <t>Rhus typhina</t>
+          <t>Rhus Typhina</t>
         </is>
       </c>
       <c r="C753" t="inlineStr">
@@ -26901,7 +26901,7 @@
       </c>
       <c r="B754" t="inlineStr">
         <is>
-          <t>Rhus typhina</t>
+          <t>Rhus Typhina</t>
         </is>
       </c>
       <c r="C754" t="inlineStr">
@@ -26934,7 +26934,7 @@
       </c>
       <c r="B755" t="inlineStr">
         <is>
-          <t>Rhus typhina</t>
+          <t>Rhus Typhina</t>
         </is>
       </c>
       <c r="C755" t="inlineStr">
@@ -26972,7 +26972,7 @@
       </c>
       <c r="B756" t="inlineStr">
         <is>
-          <t>Rhus typhina</t>
+          <t>Rhus Typhina</t>
         </is>
       </c>
       <c r="C756" t="inlineStr">
@@ -27497,7 +27497,7 @@
       </c>
       <c r="B771" t="inlineStr">
         <is>
-          <t>Salix cinerea</t>
+          <t>Salix Cinerea</t>
         </is>
       </c>
       <c r="C771" t="inlineStr">
@@ -27563,7 +27563,7 @@
       </c>
       <c r="B773" t="inlineStr">
         <is>
-          <t>Sambucus nigra</t>
+          <t>Sambucus Nigra</t>
         </is>
       </c>
       <c r="C773" t="inlineStr">
@@ -27596,7 +27596,7 @@
       </c>
       <c r="B774" t="inlineStr">
         <is>
-          <t>Sequoia sempervirens</t>
+          <t>Sequoia Sempervirens</t>
         </is>
       </c>
       <c r="C774" t="inlineStr">
@@ -27629,7 +27629,7 @@
       </c>
       <c r="B775" t="inlineStr">
         <is>
-          <t>Sequoia sempervirens</t>
+          <t>Sequoia Sempervirens</t>
         </is>
       </c>
       <c r="C775" t="inlineStr">
@@ -27662,7 +27662,7 @@
       </c>
       <c r="B776" t="inlineStr">
         <is>
-          <t>Sequoia sempervirens</t>
+          <t>Sequoia Sempervirens</t>
         </is>
       </c>
       <c r="C776" t="inlineStr">
@@ -27695,7 +27695,7 @@
       </c>
       <c r="B777" t="inlineStr">
         <is>
-          <t>Sophora japonica</t>
+          <t>Sophora Japonica</t>
         </is>
       </c>
       <c r="C777" t="inlineStr">
@@ -28159,7 +28159,7 @@
       </c>
       <c r="B790" t="inlineStr">
         <is>
-          <t>Sorbus aucuparia</t>
+          <t>Sorbus Aucuparia</t>
         </is>
       </c>
       <c r="C790" t="inlineStr">
@@ -28192,7 +28192,7 @@
       </c>
       <c r="B791" t="inlineStr">
         <is>
-          <t>Sorbus aucuparia</t>
+          <t>Sorbus Aucuparia</t>
         </is>
       </c>
       <c r="C791" t="inlineStr">
@@ -28230,7 +28230,7 @@
       </c>
       <c r="B792" t="inlineStr">
         <is>
-          <t>Sorbus aucuparia</t>
+          <t>Sorbus Aucuparia</t>
         </is>
       </c>
       <c r="C792" t="inlineStr">
@@ -28268,7 +28268,7 @@
       </c>
       <c r="B793" t="inlineStr">
         <is>
-          <t>Sorbus aucuparia</t>
+          <t>Sorbus Aucuparia</t>
         </is>
       </c>
       <c r="C793" t="inlineStr">
@@ -28306,7 +28306,7 @@
       </c>
       <c r="B794" t="inlineStr">
         <is>
-          <t>Sorbus aucuparia</t>
+          <t>Sorbus Aucuparia</t>
         </is>
       </c>
       <c r="C794" t="inlineStr">
@@ -28519,7 +28519,7 @@
       </c>
       <c r="B800" t="inlineStr">
         <is>
-          <t>Sorbus intermedia</t>
+          <t>Sorbus Intermedia</t>
         </is>
       </c>
       <c r="C800" t="inlineStr">
@@ -28552,7 +28552,7 @@
       </c>
       <c r="B801" t="inlineStr">
         <is>
-          <t>Sorbus intermedia</t>
+          <t>Sorbus Intermedia</t>
         </is>
       </c>
       <c r="C801" t="inlineStr">
@@ -28590,7 +28590,7 @@
       </c>
       <c r="B802" t="inlineStr">
         <is>
-          <t>Sorbus intermedia</t>
+          <t>Sorbus Intermedia</t>
         </is>
       </c>
       <c r="C802" t="inlineStr">
@@ -28628,7 +28628,7 @@
       </c>
       <c r="B803" t="inlineStr">
         <is>
-          <t>Sorbus pseudovilmorinii</t>
+          <t>Sorbus Pseudovilmorinii</t>
         </is>
       </c>
       <c r="C803" t="inlineStr">
@@ -28732,7 +28732,7 @@
       </c>
       <c r="B806" t="inlineStr">
         <is>
-          <t>Sorbus torminalis</t>
+          <t>Sorbus Torminalis</t>
         </is>
       </c>
       <c r="C806" t="inlineStr">
@@ -28765,7 +28765,7 @@
       </c>
       <c r="B807" t="inlineStr">
         <is>
-          <t>Sorbus torminalis</t>
+          <t>Sorbus Torminalis</t>
         </is>
       </c>
       <c r="C807" t="inlineStr">
@@ -28803,7 +28803,7 @@
       </c>
       <c r="B808" t="inlineStr">
         <is>
-          <t>Sorbus torminalis</t>
+          <t>Sorbus Torminalis</t>
         </is>
       </c>
       <c r="C808" t="inlineStr">
@@ -28836,7 +28836,7 @@
       </c>
       <c r="B809" t="inlineStr">
         <is>
-          <t>Sorbus vilmorinii</t>
+          <t>Sorbus Vilmorinii</t>
         </is>
       </c>
       <c r="C809" t="inlineStr">
@@ -28874,7 +28874,7 @@
       </c>
       <c r="B810" t="inlineStr">
         <is>
-          <t>Stewartia pseudocamellia</t>
+          <t>Stewartia Pseudocamellia</t>
         </is>
       </c>
       <c r="C810" t="inlineStr">
@@ -28940,7 +28940,7 @@
       </c>
       <c r="B812" t="inlineStr">
         <is>
-          <t>Taxodium distichum</t>
+          <t>Taxodium Distichum</t>
         </is>
       </c>
       <c r="C812" t="inlineStr">
@@ -28973,7 +28973,7 @@
       </c>
       <c r="B813" t="inlineStr">
         <is>
-          <t>Taxus baccata</t>
+          <t>Taxus Baccata</t>
         </is>
       </c>
       <c r="C813" t="inlineStr">
@@ -29006,7 +29006,7 @@
       </c>
       <c r="B814" t="inlineStr">
         <is>
-          <t>Taxus baccata</t>
+          <t>Taxus Baccata</t>
         </is>
       </c>
       <c r="C814" t="inlineStr">
@@ -29072,7 +29072,7 @@
       </c>
       <c r="B816" t="inlineStr">
         <is>
-          <t>Taxus baccata</t>
+          <t>Taxus Baccata</t>
         </is>
       </c>
       <c r="C816" t="inlineStr">
@@ -29105,7 +29105,7 @@
       </c>
       <c r="B817" t="inlineStr">
         <is>
-          <t>Tetradium daniellii</t>
+          <t>Tetradium Daniellii</t>
         </is>
       </c>
       <c r="C817" t="inlineStr">
@@ -29138,7 +29138,7 @@
       </c>
       <c r="B818" t="inlineStr">
         <is>
-          <t>Tetradium daniellii</t>
+          <t>Tetradium Daniellii</t>
         </is>
       </c>
       <c r="C818" t="inlineStr">
@@ -29303,7 +29303,7 @@
       </c>
       <c r="B823" t="inlineStr">
         <is>
-          <t>Thujopsis dolabrata</t>
+          <t>Thujopsis Dolabrata</t>
         </is>
       </c>
       <c r="C823" t="inlineStr">
@@ -29374,7 +29374,7 @@
       </c>
       <c r="B825" t="inlineStr">
         <is>
-          <t>Tilia cordata</t>
+          <t>Tilia Cordata</t>
         </is>
       </c>
       <c r="C825" t="inlineStr">
@@ -29412,7 +29412,7 @@
       </c>
       <c r="B826" t="inlineStr">
         <is>
-          <t>Tilia cordata</t>
+          <t>Tilia Cordata</t>
         </is>
       </c>
       <c r="C826" t="inlineStr">
@@ -29450,7 +29450,7 @@
       </c>
       <c r="B827" t="inlineStr">
         <is>
-          <t>Tilia cordata</t>
+          <t>Tilia Cordata</t>
         </is>
       </c>
       <c r="C827" t="inlineStr">
@@ -29488,7 +29488,7 @@
       </c>
       <c r="B828" t="inlineStr">
         <is>
-          <t>Tilia cordata</t>
+          <t>Tilia Cordata</t>
         </is>
       </c>
       <c r="C828" t="inlineStr">
@@ -29526,7 +29526,7 @@
       </c>
       <c r="B829" t="inlineStr">
         <is>
-          <t>Tilia cordata</t>
+          <t>Tilia Cordata</t>
         </is>
       </c>
       <c r="C829" t="inlineStr">
@@ -29734,7 +29734,7 @@
       </c>
       <c r="B835" t="inlineStr">
         <is>
-          <t>Tilia henryana</t>
+          <t>Tilia Henryana</t>
         </is>
       </c>
       <c r="C835" t="inlineStr">
@@ -29772,7 +29772,7 @@
       </c>
       <c r="B836" t="inlineStr">
         <is>
-          <t>Tilia platyphyllos</t>
+          <t>Tilia Platyphyllos</t>
         </is>
       </c>
       <c r="C836" t="inlineStr">
@@ -29843,7 +29843,7 @@
       </c>
       <c r="B838" t="inlineStr">
         <is>
-          <t>Tilia x</t>
+          <t>Tilia X</t>
         </is>
       </c>
       <c r="C838" t="inlineStr">
@@ -30132,7 +30132,7 @@
       </c>
       <c r="B846" t="inlineStr">
         <is>
-          <t>Toona sinensis</t>
+          <t>Toona Sinensis</t>
         </is>
       </c>
       <c r="C846" t="inlineStr">
@@ -30170,7 +30170,7 @@
       </c>
       <c r="B847" t="inlineStr">
         <is>
-          <t>Toona sinensis</t>
+          <t>Toona Sinensis</t>
         </is>
       </c>
       <c r="C847" t="inlineStr">
@@ -30203,7 +30203,7 @@
       </c>
       <c r="B848" t="inlineStr">
         <is>
-          <t>Tsuga canadensis</t>
+          <t>Tsuga Canadensis</t>
         </is>
       </c>
       <c r="C848" t="inlineStr">
@@ -30236,7 +30236,7 @@
       </c>
       <c r="B849" t="inlineStr">
         <is>
-          <t>Tsuga canadensis</t>
+          <t>Tsuga Canadensis</t>
         </is>
       </c>
       <c r="C849" t="inlineStr">
@@ -30269,7 +30269,7 @@
       </c>
       <c r="B850" t="inlineStr">
         <is>
-          <t>Tsuga heterophylla</t>
+          <t>Tsuga Heterophylla</t>
         </is>
       </c>
       <c r="C850" t="inlineStr">
@@ -30411,7 +30411,7 @@
       </c>
       <c r="B854" t="inlineStr">
         <is>
-          <t>Ulmus hollandica</t>
+          <t>Ulmus Hollandica</t>
         </is>
       </c>
       <c r="C854" t="inlineStr">
@@ -30444,7 +30444,7 @@
       </c>
       <c r="B855" t="inlineStr">
         <is>
-          <t>Ulmus minor</t>
+          <t>Ulmus Minor</t>
         </is>
       </c>
       <c r="C855" t="inlineStr">
@@ -30477,7 +30477,7 @@
       </c>
       <c r="B856" t="inlineStr">
         <is>
-          <t>Zelkova serrata</t>
+          <t>Zelkova Serrata</t>
         </is>
       </c>
       <c r="C856" t="inlineStr">
@@ -30515,7 +30515,7 @@
       </c>
       <c r="B857" t="inlineStr">
         <is>
-          <t>Zelkova serrata</t>
+          <t>Zelkova Serrata</t>
         </is>
       </c>
       <c r="C857" t="inlineStr">

</xml_diff>

<commit_message>
fix: remove logo from PDF and make Excel headers bold
- Removed logo from PDF header
- Made header row bold in Excel file
- PDF file size reduced from 230.7KB to 107.7KB
- Cleaner header layout without logo
</commit_message>
<xml_diff>
--- a/files/availability-list-2026.xlsx
+++ b/files/availability-list-2026.xlsx
@@ -17,13 +17,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -46,9 +49,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -452,42 +456,42 @@
   <sheetData>
     <row r="1" ht="85" customHeight="1"/>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>SKU</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>Botanical Name</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>Common Name</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>Pot Size</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>Height (cm)</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>Girth (cm)</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>Price (GBP)</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>Stock</t>
         </is>

</xml_diff>